<commit_message>
Update confirmation, explanation, visual md/png with rsi and head_injury; regenerate sample
</commit_message>
<xml_diff>
--- a/data dicision/field adapter/field_confirmation_table_v1.xlsx
+++ b/data dicision/field adapter/field_confirmation_table_v1.xlsx
@@ -1,30 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\vanila\code\EHR-Predict\data dicision\field adapter\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{566DA6D2-5A47-4664-B180-0A0488524D22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="field_confirmation" sheetId="1" r:id="rId1"/>
     <sheet name="color_legend" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">field_confirmation!$A$1:$M$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">field_confirmation!$A$1:$M$42</definedName>
   </definedNames>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="627" uniqueCount="313">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="560" uniqueCount="285">
   <si>
     <t>group</t>
   </si>
@@ -302,28 +296,43 @@
     <t>rsi</t>
   </si>
   <si>
-    <t>ED shock index / reverse shock index candidate</t>
-  </si>
-  <si>
-    <t>Hold formula direction</t>
+    <t>Reverse shock index</t>
   </si>
   <si>
     <t>Derived ED</t>
   </si>
   <si>
-    <t>ED heart rate and ED SBP</t>
+    <t>ED SBP / ED HR</t>
   </si>
   <si>
     <t>ratio</t>
   </si>
   <si>
-    <t>Static/pre-ICU input after formula confirmation</t>
-  </si>
-  <si>
-    <t>Formula hold</t>
-  </si>
-  <si>
-    <t>Current registry uses ED_HR / ED_SBP; confirm whether UW intended reverse SI.</t>
+    <t>Resolved: Reverse SI</t>
+  </si>
+  <si>
+    <t>rSI = SBP/HR. Confirmed from uw_fields.png.</t>
+  </si>
+  <si>
+    <t>headInjury</t>
+  </si>
+  <si>
+    <t>head_injury</t>
+  </si>
+  <si>
+    <t>Head injury indicator</t>
+  </si>
+  <si>
+    <t>Derived ICD</t>
+  </si>
+  <si>
+    <t>diagnoses_icd (S00-S09 / 800-854)</t>
+  </si>
+  <si>
+    <t>ICD broad rule</t>
+  </si>
+  <si>
+    <t>Broad rule: ICD-10 S00-S09 or ICD-9 800-804,850-854.</t>
   </si>
   <si>
     <t>er_dispCat</t>
@@ -350,37 +359,7 @@
     <t>Codebook hold</t>
   </si>
   <si>
-    <t>MIMIC C4 raw values: ADMITTED/OTHER/HOME/TRANSFER. UW values observed: 1.0/2.0. Exact UW codebook needed.</t>
-  </si>
-  <si>
-    <t>headInjury</t>
-  </si>
-  <si>
-    <t>head_injury</t>
-  </si>
-  <si>
-    <t>Head injury indicator</t>
-  </si>
-  <si>
-    <t>Recommended static proxy</t>
-  </si>
-  <si>
-    <t>Include after rule confirmation</t>
-  </si>
-  <si>
-    <t>Derived ICD diagnosis</t>
-  </si>
-  <si>
-    <t>Hospital diagnosis ICD; ED diagnosis supportive only</t>
-  </si>
-  <si>
-    <t>Static trauma attribute with provenance</t>
-  </si>
-  <si>
-    <t>ICD rule</t>
-  </si>
-  <si>
-    <t>Recommended broad rule: ICD-10 S00-S09 or ICD-9 800-804/850-854. Strict TBI alternative: ICD-10 S06 or ICD-9 850-854. E-codes are not reliable anatomy.</t>
+    <t>MIMIC C4 raw values: ADMITTED/OTHER/HOME/TRANSFER. UW: 1.0/2.0. Codebook needed.</t>
   </si>
   <si>
     <t>Initial.ED.SBPCat</t>
@@ -395,13 +374,16 @@
     <t>Hold</t>
   </si>
   <si>
-    <t>Hold until UW thresholds are known</t>
-  </si>
-  <si>
-    <t>Threshold hold</t>
-  </si>
-  <si>
-    <t>Needs UW thresholds/codebook.</t>
+    <t>Hold — threshold confirmed</t>
+  </si>
+  <si>
+    <t>Not in input; use for UW-aligned eval</t>
+  </si>
+  <si>
+    <t>Cat from 90/111</t>
+  </si>
+  <si>
+    <t>Thresholds confirmed: ≥111/90-110/≤89.</t>
   </si>
   <si>
     <t>rSICat</t>
@@ -413,6 +395,15 @@
     <t>rSI category</t>
   </si>
   <si>
+    <t>Not in input</t>
+  </si>
+  <si>
+    <t>Cat from 1.1/1.8</t>
+  </si>
+  <si>
+    <t>Thresholds confirmed: ≥1.8/1.1-1.7/≤1.0.</t>
+  </si>
+  <si>
     <t>Apache</t>
   </si>
   <si>
@@ -485,6 +476,51 @@
     <t>May appear after completed summary history covers at least 48h.</t>
   </si>
   <si>
+    <t>lactate48</t>
+  </si>
+  <si>
+    <t>lactate_48</t>
+  </si>
+  <si>
+    <t>First-48h lactate summary</t>
+  </si>
+  <si>
+    <t>labevents itemids 50813/52442/53154</t>
+  </si>
+  <si>
+    <t>mmol/L</t>
+  </si>
+  <si>
+    <t>RBC48</t>
+  </si>
+  <si>
+    <t>rbc_48</t>
+  </si>
+  <si>
+    <t>First-48h RBC transfusion volume</t>
+  </si>
+  <si>
+    <t>inputevents RBC itemids</t>
+  </si>
+  <si>
+    <t>ml</t>
+  </si>
+  <si>
+    <t>Sum volume within completed first 48h.</t>
+  </si>
+  <si>
+    <t>crys48</t>
+  </si>
+  <si>
+    <t>crys_48</t>
+  </si>
+  <si>
+    <t>First-48h crystalloid volume</t>
+  </si>
+  <si>
+    <t>inputevents crystalloid itemids</t>
+  </si>
+  <si>
     <t>baseDef48Cat</t>
   </si>
   <si>
@@ -494,25 +530,13 @@
     <t>First-48h base deficit category</t>
   </si>
   <si>
-    <t>Hold conditional category</t>
-  </si>
-  <si>
-    <t>Hold until thresholds known</t>
-  </si>
-  <si>
-    <t>lactate48</t>
-  </si>
-  <si>
-    <t>lactate_48</t>
-  </si>
-  <si>
-    <t>First-48h lactate summary</t>
-  </si>
-  <si>
-    <t>labevents itemids 50813/52442/53154</t>
-  </si>
-  <si>
-    <t>mmol/L</t>
+    <t>Not in input; UW-aligned eval</t>
+  </si>
+  <si>
+    <t>Cat from 3/6/10</t>
+  </si>
+  <si>
+    <t>Thresholds confirmed.</t>
   </si>
   <si>
     <t>lactate48Cat</t>
@@ -524,34 +548,7 @@
     <t>First-48h lactate category</t>
   </si>
   <si>
-    <t>RBC48</t>
-  </si>
-  <si>
-    <t>rbc_48</t>
-  </si>
-  <si>
-    <t>First-48h RBC transfusion volume</t>
-  </si>
-  <si>
-    <t>inputevents RBC itemids</t>
-  </si>
-  <si>
-    <t>ml</t>
-  </si>
-  <si>
-    <t>Sum volume within completed first 48h.</t>
-  </si>
-  <si>
-    <t>crys48</t>
-  </si>
-  <si>
-    <t>crys_48</t>
-  </si>
-  <si>
-    <t>First-48h crystalloid volume</t>
-  </si>
-  <si>
-    <t>inputevents crystalloid itemids</t>
+    <t>Cat from 3.0/5.0</t>
   </si>
   <si>
     <t>crys48Cat</t>
@@ -563,6 +560,9 @@
     <t>First-48h crystalloid category</t>
   </si>
   <si>
+    <t>Cat from 2000/5000/10000</t>
+  </si>
+  <si>
     <t>abx48</t>
   </si>
   <si>
@@ -731,57 +731,6 @@
     <t>Days in surgery, not operation count.</t>
   </si>
   <si>
-    <t>-</t>
-  </si>
-  <si>
-    <t>iv_fluid_ml_1h</t>
-  </si>
-  <si>
-    <t>Hourly crystalloid implementation variable</t>
-  </si>
-  <si>
-    <t>Intermediate</t>
-  </si>
-  <si>
-    <t>Intermediate only</t>
-  </si>
-  <si>
-    <t>ml/h</t>
-  </si>
-  <si>
-    <t>Compute bolusSum</t>
-  </si>
-  <si>
-    <t>Compute only</t>
-  </si>
-  <si>
-    <t>Not a UW final field.</t>
-  </si>
-  <si>
-    <t>rbc_ml_1h</t>
-  </si>
-  <si>
-    <t>Hourly RBC implementation variable</t>
-  </si>
-  <si>
-    <t>Compute RBCsum</t>
-  </si>
-  <si>
-    <t>surgery_hours_1h</t>
-  </si>
-  <si>
-    <t>Hourly surgery implementation variable</t>
-  </si>
-  <si>
-    <t>procedureevents/transfers OR intervals</t>
-  </si>
-  <si>
-    <t>h/h</t>
-  </si>
-  <si>
-    <t>Compute surgHours/surgSum</t>
-  </si>
-  <si>
     <t>G4</t>
   </si>
   <si>
@@ -806,18 +755,6 @@
     <t>Latest value at or before h.</t>
   </si>
   <si>
-    <t>acidosisCat</t>
-  </si>
-  <si>
-    <t>acidosis_cat</t>
-  </si>
-  <si>
-    <t>Acidosis category</t>
-  </si>
-  <si>
-    <t>bicarb/base_excess</t>
-  </si>
-  <si>
     <t>StrongIon</t>
   </si>
   <si>
@@ -875,22 +812,19 @@
     <t>lymphocytes</t>
   </si>
   <si>
-    <t>Lymphocyte percentage</t>
+    <t>Absolute lymphocyte count</t>
   </si>
   <si>
     <t>labevents itemids 51244/51245/51690</t>
   </si>
   <si>
-    <t>%</t>
-  </si>
-  <si>
-    <t>Use percent only; do not silently merge absolute counts.</t>
+    <t>Convert from % to K/uL via same-time WBC if needed.</t>
   </si>
   <si>
     <t>neutrophils</t>
   </si>
   <si>
-    <t>Neutrophil percentage</t>
+    <t>Absolute neutrophil count</t>
   </si>
   <si>
     <t>labevents itemid 51256</t>
@@ -908,33 +842,15 @@
     <t>outputevents urine itemids</t>
   </si>
   <si>
+    <t>mL/h</t>
+  </si>
+  <si>
     <t>G4 output with observed metadata</t>
   </si>
   <si>
     <t>Hourly sum, split intervals carefully.</t>
   </si>
   <si>
-    <t>na/k/cl/base_excess/lactate</t>
-  </si>
-  <si>
-    <t>Intermediate laboratory variables</t>
-  </si>
-  <si>
-    <t>labevents/chartevents</t>
-  </si>
-  <si>
-    <t>various</t>
-  </si>
-  <si>
-    <t>Compute StrongIon/baseDef48/lactate48/acidosisCat</t>
-  </si>
-  <si>
-    <t>Not mainline final inputs unless explicitly selected for ablation.</t>
-  </si>
-  <si>
-    <t>group/color</t>
-  </si>
-  <si>
     <t>meaning</t>
   </si>
   <si>
@@ -944,32 +860,26 @@
     <t>Static / pre-ICU</t>
   </si>
   <si>
-    <t>First-48h conditional summary fields</t>
-  </si>
-  <si>
-    <t>Treatment/exposure</t>
-  </si>
-  <si>
-    <t>Labs/output</t>
-  </si>
-  <si>
-    <t>VENT</t>
-  </si>
-  <si>
-    <t>Ventilation-highlighted fields</t>
+    <t>First-48h summary</t>
+  </si>
+  <si>
+    <t>Treatment / exposure</t>
+  </si>
+  <si>
+    <t>Labs / output</t>
   </si>
   <si>
     <t>EXCLUDE</t>
   </si>
   <si>
-    <t>Excluded field</t>
+    <t>Excluded</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -985,16 +895,8 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="10">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1039,12 +941,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF9999"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFFDEADA"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -1077,7 +973,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1100,42 +996,19 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1173,7 +1046,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -1207,7 +1080,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -1242,10 +1114,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1418,26 +1289,26 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M47"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M42"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="8.7265625" customWidth="1"/>
-    <col min="2" max="2" width="18.7265625" customWidth="1"/>
-    <col min="3" max="3" width="24.7265625" customWidth="1"/>
-    <col min="4" max="4" width="26.7265625" customWidth="1"/>
-    <col min="5" max="5" width="24.7265625" customWidth="1"/>
-    <col min="6" max="6" width="22.7265625" customWidth="1"/>
-    <col min="7" max="7" width="24.7265625" customWidth="1"/>
-    <col min="8" max="8" width="48.7265625" customWidth="1"/>
-    <col min="9" max="9" width="12.7265625" customWidth="1"/>
-    <col min="10" max="10" width="22.7265625" customWidth="1"/>
-    <col min="11" max="11" width="38.7265625" customWidth="1"/>
-    <col min="12" max="12" width="14.7265625" customWidth="1"/>
-    <col min="13" max="13" width="52.7265625" customWidth="1"/>
+    <col min="1" max="1" width="8.7109375" customWidth="1"/>
+    <col min="2" max="2" width="18.7109375" customWidth="1"/>
+    <col min="3" max="3" width="24.7109375" customWidth="1"/>
+    <col min="4" max="4" width="26.7109375" customWidth="1"/>
+    <col min="5" max="5" width="24.7109375" customWidth="1"/>
+    <col min="6" max="6" width="22.7109375" customWidth="1"/>
+    <col min="7" max="7" width="24.7109375" customWidth="1"/>
+    <col min="8" max="8" width="48.7109375" customWidth="1"/>
+    <col min="9" max="9" width="12.7109375" customWidth="1"/>
+    <col min="10" max="10" width="22.7109375" customWidth="1"/>
+    <col min="11" max="11" width="38.7109375" customWidth="1"/>
+    <col min="12" max="12" width="14.7109375" customWidth="1"/>
+    <col min="13" max="13" width="52.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:13">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1478,7 +1349,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="29" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:13">
       <c r="A2" s="2" t="s">
         <v>13</v>
       </c>
@@ -1494,7 +1365,7 @@
       <c r="E2" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="F2" s="9" t="s">
+      <c r="F2" s="2" t="s">
         <v>17</v>
       </c>
       <c r="G2" s="2" t="s">
@@ -1519,7 +1390,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="29" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:13">
       <c r="A3" s="2" t="s">
         <v>13</v>
       </c>
@@ -1535,7 +1406,7 @@
       <c r="E3" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="F3" s="9" t="s">
+      <c r="F3" s="2" t="s">
         <v>17</v>
       </c>
       <c r="G3" s="2" t="s">
@@ -1560,7 +1431,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="29" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:13">
       <c r="A4" s="2" t="s">
         <v>13</v>
       </c>
@@ -1576,7 +1447,7 @@
       <c r="E4" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="F4" s="9" t="s">
+      <c r="F4" s="2" t="s">
         <v>17</v>
       </c>
       <c r="G4" s="2" t="s">
@@ -1601,7 +1472,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:13" ht="29" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:13">
       <c r="A5" s="2" t="s">
         <v>13</v>
       </c>
@@ -1617,7 +1488,7 @@
       <c r="E5" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="F5" s="9" t="s">
+      <c r="F5" s="2" t="s">
         <v>17</v>
       </c>
       <c r="G5" s="2" t="s">
@@ -1642,7 +1513,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:13" ht="29" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:13">
       <c r="A6" s="2" t="s">
         <v>13</v>
       </c>
@@ -1658,7 +1529,7 @@
       <c r="E6" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="F6" s="9" t="s">
+      <c r="F6" s="2" t="s">
         <v>17</v>
       </c>
       <c r="G6" s="2" t="s">
@@ -1683,7 +1554,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="7" spans="1:13" ht="29" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:13">
       <c r="A7" s="2" t="s">
         <v>13</v>
       </c>
@@ -1699,7 +1570,7 @@
       <c r="E7" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="F7" s="9" t="s">
+      <c r="F7" s="2" t="s">
         <v>17</v>
       </c>
       <c r="G7" s="2" t="s">
@@ -1724,7 +1595,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="8" spans="1:13" ht="29" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:13">
       <c r="A8" s="2" t="s">
         <v>13</v>
       </c>
@@ -1740,7 +1611,7 @@
       <c r="E8" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="F8" s="9" t="s">
+      <c r="F8" s="2" t="s">
         <v>17</v>
       </c>
       <c r="G8" s="2" t="s">
@@ -1765,7 +1636,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:13">
       <c r="A9" s="3" t="s">
         <v>49</v>
       </c>
@@ -1781,7 +1652,7 @@
       <c r="E9" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="F9" s="10" t="s">
+      <c r="F9" s="3" t="s">
         <v>17</v>
       </c>
       <c r="G9" s="3" t="s">
@@ -1806,7 +1677,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:13">
       <c r="A10" s="3" t="s">
         <v>49</v>
       </c>
@@ -1822,7 +1693,7 @@
       <c r="E10" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="F10" s="10" t="s">
+      <c r="F10" s="3" t="s">
         <v>17</v>
       </c>
       <c r="G10" s="3" t="s">
@@ -1847,7 +1718,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:13">
       <c r="A11" s="3" t="s">
         <v>49</v>
       </c>
@@ -1863,7 +1734,7 @@
       <c r="E11" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="F11" s="10" t="s">
+      <c r="F11" s="3" t="s">
         <v>17</v>
       </c>
       <c r="G11" s="3" t="s">
@@ -1888,7 +1759,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="12" spans="1:13" ht="29" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:13">
       <c r="A12" s="3" t="s">
         <v>49</v>
       </c>
@@ -1904,7 +1775,7 @@
       <c r="E12" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="F12" s="10" t="s">
+      <c r="F12" s="3" t="s">
         <v>17</v>
       </c>
       <c r="G12" s="3" t="s">
@@ -1929,7 +1800,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="13" spans="1:13" ht="29" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:13">
       <c r="A13" s="3" t="s">
         <v>49</v>
       </c>
@@ -1945,7 +1816,7 @@
       <c r="E13" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="F13" s="10" t="s">
+      <c r="F13" s="3" t="s">
         <v>17</v>
       </c>
       <c r="G13" s="3" t="s">
@@ -1970,7 +1841,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="14" spans="1:13" ht="29" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:13">
       <c r="A14" s="3" t="s">
         <v>49</v>
       </c>
@@ -1987,130 +1858,130 @@
         <v>76</v>
       </c>
       <c r="F14" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="G14" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="G14" s="3" t="s">
+      <c r="H14" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="H14" s="3" t="s">
+      <c r="I14" s="3" t="s">
         <v>95</v>
-      </c>
-      <c r="I14" s="3" t="s">
-        <v>96</v>
       </c>
       <c r="J14" s="3" t="s">
         <v>80</v>
       </c>
       <c r="K14" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="L14" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="M14" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="L14" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="M14" s="3" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13" ht="29" x14ac:dyDescent="0.35">
+    </row>
+    <row r="15" spans="1:13">
       <c r="A15" s="3" t="s">
         <v>49</v>
       </c>
       <c r="B15" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="D15" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="E15" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="G15" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="H15" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="E15" s="3" t="s">
+      <c r="I15" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="J15" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="K15" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="L15" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="F15" s="3" t="s">
+      <c r="M15" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="G15" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="H15" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="I15" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="J15" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="K15" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="L15" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="M15" s="3" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="16" spans="1:13" ht="43.5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="16" spans="1:13">
       <c r="A16" s="3" t="s">
         <v>49</v>
       </c>
       <c r="B16" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="F16" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="G16" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="H16" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="I16" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="J16" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="K16" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="E16" s="3" t="s">
+      <c r="L16" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="F16" s="3" t="s">
+      <c r="M16" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="G16" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="H16" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="I16" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="J16" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="K16" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="L16" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="M16" s="3" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
+    </row>
+    <row r="17" spans="1:13">
       <c r="A17" s="3" t="s">
         <v>49</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>103</v>
+        <v>117</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="G17" s="3" t="s">
         <v>68</v>
@@ -2125,33 +1996,33 @@
         <v>80</v>
       </c>
       <c r="K17" s="3" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="L17" s="3" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="M17" s="3" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13">
       <c r="A18" s="3" t="s">
         <v>49</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>103</v>
+        <v>117</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="G18" s="3" t="s">
         <v>68</v>
@@ -2166,182 +2037,182 @@
         <v>80</v>
       </c>
       <c r="K18" s="3" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="L18" s="3" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="M18" s="3" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="19" spans="1:13" ht="29" x14ac:dyDescent="0.35">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13">
       <c r="A19" s="4" t="s">
         <v>49</v>
       </c>
       <c r="B19" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="C19" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="C19" s="4" t="s">
+      <c r="D19" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="D19" s="4" t="s">
+      <c r="E19" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="E19" s="4" t="s">
+      <c r="F19" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="G19" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="F19" s="4" t="s">
-        <v>132</v>
-      </c>
-      <c r="G19" s="4" t="s">
+      <c r="H19" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="H19" s="4" t="s">
+      <c r="I19" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="I19" s="4" t="s">
+      <c r="J19" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="J19" s="4" t="s">
+      <c r="K19" s="4" t="s">
         <v>136</v>
       </c>
-      <c r="K19" s="4" t="s">
+      <c r="L19" s="4" t="s">
         <v>137</v>
       </c>
-      <c r="L19" s="4" t="s">
+      <c r="M19" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="M19" s="4" t="s">
+    </row>
+    <row r="20" spans="1:13">
+      <c r="A20" s="5" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="20" spans="1:13" ht="29" x14ac:dyDescent="0.35">
-      <c r="A20" s="5" t="s">
+      <c r="B20" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="C20" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="C20" s="5" t="s">
+      <c r="D20" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="D20" s="5" t="s">
+      <c r="E20" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="E20" s="5" t="s">
+      <c r="F20" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="F20" s="5" t="s">
+      <c r="G20" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="G20" s="5" t="s">
+      <c r="H20" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="H20" s="5" t="s">
+      <c r="I20" s="5" t="s">
         <v>147</v>
       </c>
-      <c r="I20" s="5" t="s">
+      <c r="J20" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="J20" s="5" t="s">
+      <c r="K20" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="K20" s="5" t="s">
+      <c r="L20" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="L20" s="5" t="s">
+      <c r="M20" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="M20" s="5" t="s">
+    </row>
+    <row r="21" spans="1:13">
+      <c r="A21" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="B21" s="5" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A21" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="B21" s="5" t="s">
+      <c r="C21" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="C21" s="5" t="s">
+      <c r="D21" s="5" t="s">
         <v>154</v>
       </c>
-      <c r="D21" s="5" t="s">
+      <c r="E21" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="F21" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="G21" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="H21" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="E21" s="5" t="s">
+      <c r="I21" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="F21" s="5" t="s">
-        <v>122</v>
-      </c>
-      <c r="G21" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="H21" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="I21" s="5" t="s">
-        <v>79</v>
-      </c>
       <c r="J21" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="K21" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="K21" s="5" t="s">
+      <c r="L21" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="M21" s="5" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13">
+      <c r="A22" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="B22" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="L21" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="M21" s="5" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="22" spans="1:13" ht="29" x14ac:dyDescent="0.35">
-      <c r="A22" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="B22" s="5" t="s">
+      <c r="C22" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="C22" s="5" t="s">
+      <c r="D22" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="D22" s="5" t="s">
-        <v>160</v>
-      </c>
       <c r="E22" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="F22" s="5" t="s">
         <v>144</v>
-      </c>
-      <c r="F22" s="5" t="s">
-        <v>145</v>
       </c>
       <c r="G22" s="5" t="s">
         <v>53</v>
       </c>
       <c r="H22" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="I22" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="I22" s="5" t="s">
+      <c r="J22" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="K22" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="L22" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="M22" s="5" t="s">
         <v>162</v>
       </c>
-      <c r="J22" s="5" t="s">
-        <v>149</v>
-      </c>
-      <c r="K22" s="5" t="s">
-        <v>150</v>
-      </c>
-      <c r="L22" s="5" t="s">
-        <v>151</v>
-      </c>
-      <c r="M22" s="5" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
+    </row>
+    <row r="23" spans="1:13">
       <c r="A23" s="5" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B23" s="5" t="s">
         <v>163</v>
@@ -2353,1094 +2224,881 @@
         <v>165</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>156</v>
+        <v>143</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>122</v>
+        <v>144</v>
       </c>
       <c r="G23" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="H23" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="I23" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="J23" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="K23" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="L23" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="M23" s="5" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13">
+      <c r="A24" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>167</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>168</v>
+      </c>
+      <c r="D24" s="5" t="s">
+        <v>169</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="F24" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="G24" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="H23" s="5" t="s">
-        <v>159</v>
-      </c>
-      <c r="I23" s="5" t="s">
+      <c r="H24" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="I24" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="J23" s="5" t="s">
-        <v>149</v>
-      </c>
-      <c r="K23" s="5" t="s">
-        <v>157</v>
-      </c>
-      <c r="L23" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="M23" s="5" t="s">
+      <c r="J24" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="K24" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="L24" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="M24" s="5" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13">
+      <c r="A25" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="D25" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="F25" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="G25" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="H25" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="I25" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="J25" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="K25" s="5" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="24" spans="1:13" ht="29" x14ac:dyDescent="0.35">
-      <c r="A24" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="B24" s="5" t="s">
-        <v>166</v>
-      </c>
-      <c r="C24" s="5" t="s">
-        <v>167</v>
-      </c>
-      <c r="D24" s="5" t="s">
-        <v>168</v>
-      </c>
-      <c r="E24" s="5" t="s">
-        <v>144</v>
-      </c>
-      <c r="F24" s="5" t="s">
-        <v>145</v>
-      </c>
-      <c r="G24" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="H24" s="5" t="s">
-        <v>169</v>
-      </c>
-      <c r="I24" s="5" t="s">
-        <v>170</v>
-      </c>
-      <c r="J24" s="5" t="s">
-        <v>149</v>
-      </c>
-      <c r="K24" s="5" t="s">
-        <v>150</v>
-      </c>
-      <c r="L24" s="5" t="s">
-        <v>151</v>
-      </c>
-      <c r="M24" s="5" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A25" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="B25" s="5" t="s">
+      <c r="L25" s="5" t="s">
+        <v>176</v>
+      </c>
+      <c r="M25" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="C25" s="5" t="s">
-        <v>173</v>
-      </c>
-      <c r="D25" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="E25" s="5" t="s">
-        <v>144</v>
-      </c>
-      <c r="F25" s="5" t="s">
-        <v>145</v>
-      </c>
-      <c r="G25" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="H25" s="5" t="s">
-        <v>175</v>
-      </c>
-      <c r="I25" s="5" t="s">
-        <v>170</v>
-      </c>
-      <c r="J25" s="5" t="s">
-        <v>149</v>
-      </c>
-      <c r="K25" s="5" t="s">
-        <v>150</v>
-      </c>
-      <c r="L25" s="5" t="s">
-        <v>151</v>
-      </c>
-      <c r="M25" s="5" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
+    </row>
+    <row r="26" spans="1:13">
       <c r="A26" s="5" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>156</v>
+        <v>117</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="G26" s="5" t="s">
         <v>68</v>
       </c>
       <c r="H26" s="5" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="I26" s="5" t="s">
         <v>79</v>
       </c>
       <c r="J26" s="5" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="K26" s="5" t="s">
-        <v>157</v>
+        <v>125</v>
       </c>
       <c r="L26" s="5" t="s">
-        <v>124</v>
+        <v>180</v>
       </c>
       <c r="M26" s="5" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.35">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13">
       <c r="A27" s="5" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="I27" s="5" t="s">
         <v>63</v>
       </c>
       <c r="J27" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="K27" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="K27" s="5" t="s">
-        <v>150</v>
-      </c>
       <c r="L27" s="5" t="s">
+        <v>187</v>
+      </c>
+      <c r="M27" s="5" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13">
+      <c r="A28" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="D28" s="5" t="s">
+        <v>191</v>
+      </c>
+      <c r="E28" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="F28" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="G28" s="5" t="s">
         <v>185</v>
       </c>
-      <c r="M27" s="5" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A28" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="B28" s="5" t="s">
-        <v>187</v>
-      </c>
-      <c r="C28" s="5" t="s">
-        <v>188</v>
-      </c>
-      <c r="D28" s="5" t="s">
-        <v>189</v>
-      </c>
-      <c r="E28" s="5" t="s">
-        <v>144</v>
-      </c>
-      <c r="F28" s="5" t="s">
-        <v>182</v>
-      </c>
-      <c r="G28" s="5" t="s">
-        <v>183</v>
-      </c>
       <c r="H28" s="5" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="I28" s="5" t="s">
         <v>63</v>
       </c>
       <c r="J28" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="K28" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="K28" s="5" t="s">
-        <v>150</v>
-      </c>
       <c r="L28" s="5" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="M28" s="5" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="29" spans="1:13" ht="29" x14ac:dyDescent="0.35">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13">
       <c r="A29" s="6" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>197</v>
-      </c>
-      <c r="F29" s="11" t="s">
+        <v>199</v>
+      </c>
+      <c r="F29" s="6" t="s">
         <v>17</v>
       </c>
       <c r="G29" s="6" t="s">
         <v>68</v>
       </c>
       <c r="H29" s="6" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="I29" s="6" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="J29" s="6" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="K29" s="6" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="L29" s="6" t="s">
         <v>72</v>
       </c>
       <c r="M29" s="6" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="30" spans="1:13" ht="29" x14ac:dyDescent="0.35">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13">
       <c r="A30" s="6" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>197</v>
-      </c>
-      <c r="F30" s="11" t="s">
+        <v>199</v>
+      </c>
+      <c r="F30" s="6" t="s">
         <v>17</v>
       </c>
       <c r="G30" s="6" t="s">
         <v>68</v>
       </c>
       <c r="H30" s="6" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="I30" s="6" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="J30" s="6" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="K30" s="6" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="L30" s="6" t="s">
         <v>72</v>
       </c>
       <c r="M30" s="6" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13">
+      <c r="A31" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>209</v>
+      </c>
+      <c r="D31" s="6" t="s">
+        <v>210</v>
+      </c>
+      <c r="E31" s="6" t="s">
+        <v>211</v>
+      </c>
+      <c r="F31" s="6" t="s">
+        <v>212</v>
+      </c>
+      <c r="G31" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="H31" s="6" t="s">
+        <v>213</v>
+      </c>
+      <c r="I31" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="J31" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="K31" s="6" t="s">
+        <v>214</v>
+      </c>
+      <c r="L31" s="6" t="s">
+        <v>215</v>
+      </c>
+      <c r="M31" s="6" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13">
+      <c r="A32" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="B32" s="6" t="s">
+        <v>217</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>218</v>
+      </c>
+      <c r="D32" s="6" t="s">
+        <v>219</v>
+      </c>
+      <c r="E32" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="F32" s="6" t="s">
+        <v>212</v>
+      </c>
+      <c r="G32" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="H32" s="6" t="s">
+        <v>221</v>
+      </c>
+      <c r="I32" s="6" t="s">
+        <v>222</v>
+      </c>
+      <c r="J32" s="6" t="s">
         <v>201</v>
       </c>
-    </row>
-    <row r="31" spans="1:13" ht="29" x14ac:dyDescent="0.35">
-      <c r="A31" s="7" t="s">
+      <c r="K32" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="L32" s="6" t="s">
+        <v>215</v>
+      </c>
+      <c r="M32" s="6" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13">
+      <c r="A33" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>225</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>226</v>
+      </c>
+      <c r="D33" s="6" t="s">
+        <v>227</v>
+      </c>
+      <c r="E33" s="6" t="s">
+        <v>199</v>
+      </c>
+      <c r="F33" s="6" t="s">
+        <v>228</v>
+      </c>
+      <c r="G33" s="6" t="s">
+        <v>229</v>
+      </c>
+      <c r="H33" s="6" t="s">
+        <v>230</v>
+      </c>
+      <c r="I33" s="6" t="s">
+        <v>231</v>
+      </c>
+      <c r="J33" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="K33" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="L33" s="6" t="s">
         <v>193</v>
       </c>
-      <c r="B31" s="7" t="s">
-        <v>206</v>
-      </c>
-      <c r="C31" s="7" t="s">
-        <v>207</v>
-      </c>
-      <c r="D31" s="7" t="s">
-        <v>208</v>
-      </c>
-      <c r="E31" s="7" t="s">
-        <v>209</v>
-      </c>
-      <c r="F31" s="7" t="s">
-        <v>210</v>
-      </c>
-      <c r="G31" s="7" t="s">
+      <c r="M33" s="6" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13">
+      <c r="A34" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="B34" s="6" t="s">
+        <v>232</v>
+      </c>
+      <c r="C34" s="6" t="s">
+        <v>233</v>
+      </c>
+      <c r="D34" s="6" t="s">
+        <v>234</v>
+      </c>
+      <c r="E34" s="6" t="s">
+        <v>199</v>
+      </c>
+      <c r="F34" s="6" t="s">
+        <v>228</v>
+      </c>
+      <c r="G34" s="6" t="s">
+        <v>229</v>
+      </c>
+      <c r="H34" s="6" t="s">
+        <v>235</v>
+      </c>
+      <c r="I34" s="6" t="s">
+        <v>222</v>
+      </c>
+      <c r="J34" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="K34" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="L34" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="M34" s="6" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13">
+      <c r="A35" s="7" t="s">
+        <v>237</v>
+      </c>
+      <c r="B35" s="7" t="s">
+        <v>238</v>
+      </c>
+      <c r="C35" s="7" t="s">
+        <v>238</v>
+      </c>
+      <c r="D35" s="7" t="s">
+        <v>239</v>
+      </c>
+      <c r="E35" s="7" t="s">
+        <v>240</v>
+      </c>
+      <c r="F35" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="G35" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="H35" s="7" t="s">
+        <v>241</v>
+      </c>
+      <c r="I35" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="J35" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="K35" s="7" t="s">
+        <v>243</v>
+      </c>
+      <c r="L35" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="M35" s="7" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13">
+      <c r="A36" s="7" t="s">
+        <v>237</v>
+      </c>
+      <c r="B36" s="7" t="s">
+        <v>245</v>
+      </c>
+      <c r="C36" s="7" t="s">
+        <v>246</v>
+      </c>
+      <c r="D36" s="7" t="s">
+        <v>247</v>
+      </c>
+      <c r="E36" s="7" t="s">
+        <v>248</v>
+      </c>
+      <c r="F36" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="G36" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="H36" s="7" t="s">
+        <v>249</v>
+      </c>
+      <c r="I36" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="J36" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="K36" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="L36" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="M36" s="7" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13">
+      <c r="A37" s="7" t="s">
+        <v>237</v>
+      </c>
+      <c r="B37" s="7" t="s">
+        <v>252</v>
+      </c>
+      <c r="C37" s="7" t="s">
+        <v>252</v>
+      </c>
+      <c r="D37" s="7" t="s">
+        <v>253</v>
+      </c>
+      <c r="E37" s="7" t="s">
+        <v>240</v>
+      </c>
+      <c r="F37" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="G37" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="H37" s="7" t="s">
+        <v>254</v>
+      </c>
+      <c r="I37" s="7" t="s">
+        <v>255</v>
+      </c>
+      <c r="J37" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="K37" s="7" t="s">
+        <v>243</v>
+      </c>
+      <c r="L37" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="M37" s="7" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="38" spans="1:13">
+      <c r="A38" s="7" t="s">
+        <v>237</v>
+      </c>
+      <c r="B38" s="7" t="s">
+        <v>256</v>
+      </c>
+      <c r="C38" s="7" t="s">
+        <v>256</v>
+      </c>
+      <c r="D38" s="7" t="s">
+        <v>257</v>
+      </c>
+      <c r="E38" s="7" t="s">
+        <v>240</v>
+      </c>
+      <c r="F38" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="G38" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="H38" s="7" t="s">
+        <v>258</v>
+      </c>
+      <c r="I38" s="7" t="s">
+        <v>255</v>
+      </c>
+      <c r="J38" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="K38" s="7" t="s">
+        <v>243</v>
+      </c>
+      <c r="L38" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="M38" s="7" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="39" spans="1:13">
+      <c r="A39" s="7" t="s">
+        <v>237</v>
+      </c>
+      <c r="B39" s="7" t="s">
+        <v>259</v>
+      </c>
+      <c r="C39" s="7" t="s">
+        <v>259</v>
+      </c>
+      <c r="D39" s="7" t="s">
+        <v>260</v>
+      </c>
+      <c r="E39" s="7" t="s">
+        <v>240</v>
+      </c>
+      <c r="F39" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="G39" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="H39" s="7" t="s">
+        <v>261</v>
+      </c>
+      <c r="I39" s="7" t="s">
+        <v>262</v>
+      </c>
+      <c r="J39" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="K39" s="7" t="s">
+        <v>243</v>
+      </c>
+      <c r="L39" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="M39" s="7" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="40" spans="1:13">
+      <c r="A40" s="7" t="s">
+        <v>237</v>
+      </c>
+      <c r="B40" s="7" t="s">
+        <v>263</v>
+      </c>
+      <c r="C40" s="7" t="s">
+        <v>263</v>
+      </c>
+      <c r="D40" s="7" t="s">
+        <v>264</v>
+      </c>
+      <c r="E40" s="7" t="s">
+        <v>240</v>
+      </c>
+      <c r="F40" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="G40" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="H40" s="7" t="s">
+        <v>265</v>
+      </c>
+      <c r="I40" s="7" t="s">
+        <v>262</v>
+      </c>
+      <c r="J40" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="K40" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="L40" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="M40" s="7" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="41" spans="1:13">
+      <c r="A41" s="7" t="s">
+        <v>237</v>
+      </c>
+      <c r="B41" s="7" t="s">
+        <v>267</v>
+      </c>
+      <c r="C41" s="7" t="s">
+        <v>267</v>
+      </c>
+      <c r="D41" s="7" t="s">
+        <v>268</v>
+      </c>
+      <c r="E41" s="7" t="s">
+        <v>240</v>
+      </c>
+      <c r="F41" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="G41" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="H41" s="7" t="s">
+        <v>269</v>
+      </c>
+      <c r="I41" s="7" t="s">
+        <v>262</v>
+      </c>
+      <c r="J41" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="K41" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="L41" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="M41" s="7" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="42" spans="1:13">
+      <c r="A42" s="7" t="s">
+        <v>237</v>
+      </c>
+      <c r="B42" s="7" t="s">
+        <v>270</v>
+      </c>
+      <c r="C42" s="7" t="s">
+        <v>270</v>
+      </c>
+      <c r="D42" s="7" t="s">
+        <v>271</v>
+      </c>
+      <c r="E42" s="7" t="s">
+        <v>272</v>
+      </c>
+      <c r="F42" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="G42" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="H31" s="7" t="s">
-        <v>211</v>
-      </c>
-      <c r="I31" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="J31" s="7" t="s">
+      <c r="H42" s="7" t="s">
+        <v>273</v>
+      </c>
+      <c r="I42" s="7" t="s">
+        <v>274</v>
+      </c>
+      <c r="J42" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="K31" s="7" t="s">
-        <v>212</v>
-      </c>
-      <c r="L31" s="7" t="s">
-        <v>213</v>
-      </c>
-      <c r="M31" s="7" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="32" spans="1:13" ht="29" x14ac:dyDescent="0.35">
-      <c r="A32" s="7" t="s">
-        <v>193</v>
-      </c>
-      <c r="B32" s="7" t="s">
-        <v>215</v>
-      </c>
-      <c r="C32" s="7" t="s">
-        <v>216</v>
-      </c>
-      <c r="D32" s="7" t="s">
-        <v>217</v>
-      </c>
-      <c r="E32" s="7" t="s">
-        <v>218</v>
-      </c>
-      <c r="F32" s="7" t="s">
-        <v>210</v>
-      </c>
-      <c r="G32" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="H32" s="7" t="s">
-        <v>219</v>
-      </c>
-      <c r="I32" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="J32" s="7" t="s">
-        <v>199</v>
-      </c>
-      <c r="K32" s="7" t="s">
-        <v>221</v>
-      </c>
-      <c r="L32" s="7" t="s">
-        <v>213</v>
-      </c>
-      <c r="M32" s="7" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A33" s="6" t="s">
-        <v>193</v>
-      </c>
-      <c r="B33" s="6" t="s">
-        <v>223</v>
-      </c>
-      <c r="C33" s="6" t="s">
-        <v>224</v>
-      </c>
-      <c r="D33" s="6" t="s">
-        <v>225</v>
-      </c>
-      <c r="E33" s="6" t="s">
-        <v>197</v>
-      </c>
-      <c r="F33" s="6" t="s">
-        <v>226</v>
-      </c>
-      <c r="G33" s="6" t="s">
-        <v>227</v>
-      </c>
-      <c r="H33" s="6" t="s">
-        <v>228</v>
-      </c>
-      <c r="I33" s="6" t="s">
-        <v>229</v>
-      </c>
-      <c r="J33" s="6" t="s">
-        <v>199</v>
-      </c>
-      <c r="K33" s="6" t="s">
-        <v>200</v>
-      </c>
-      <c r="L33" s="6" t="s">
-        <v>191</v>
-      </c>
-      <c r="M33" s="6" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A34" s="6" t="s">
-        <v>193</v>
-      </c>
-      <c r="B34" s="6" t="s">
-        <v>230</v>
-      </c>
-      <c r="C34" s="6" t="s">
-        <v>231</v>
-      </c>
-      <c r="D34" s="6" t="s">
-        <v>232</v>
-      </c>
-      <c r="E34" s="6" t="s">
-        <v>197</v>
-      </c>
-      <c r="F34" s="6" t="s">
-        <v>226</v>
-      </c>
-      <c r="G34" s="6" t="s">
-        <v>227</v>
-      </c>
-      <c r="H34" s="6" t="s">
-        <v>233</v>
-      </c>
-      <c r="I34" s="6" t="s">
-        <v>220</v>
-      </c>
-      <c r="J34" s="6" t="s">
-        <v>199</v>
-      </c>
-      <c r="K34" s="6" t="s">
-        <v>200</v>
-      </c>
-      <c r="L34" s="6" t="s">
-        <v>191</v>
-      </c>
-      <c r="M34" s="6" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="35" spans="1:13" ht="29" x14ac:dyDescent="0.35">
-      <c r="A35" s="6" t="s">
-        <v>193</v>
-      </c>
-      <c r="B35" s="6" t="s">
-        <v>235</v>
-      </c>
-      <c r="C35" s="6" t="s">
-        <v>236</v>
-      </c>
-      <c r="D35" s="6" t="s">
-        <v>237</v>
-      </c>
-      <c r="E35" s="6" t="s">
-        <v>238</v>
-      </c>
-      <c r="F35" s="6" t="s">
-        <v>239</v>
-      </c>
-      <c r="G35" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="H35" s="6" t="s">
-        <v>175</v>
-      </c>
-      <c r="I35" s="6" t="s">
-        <v>240</v>
-      </c>
-      <c r="J35" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="K35" s="6" t="s">
-        <v>241</v>
-      </c>
-      <c r="L35" s="6" t="s">
-        <v>242</v>
-      </c>
-      <c r="M35" s="6" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="36" spans="1:13" ht="29" x14ac:dyDescent="0.35">
-      <c r="A36" s="6" t="s">
-        <v>193</v>
-      </c>
-      <c r="B36" s="6" t="s">
-        <v>235</v>
-      </c>
-      <c r="C36" s="6" t="s">
-        <v>244</v>
-      </c>
-      <c r="D36" s="6" t="s">
-        <v>245</v>
-      </c>
-      <c r="E36" s="6" t="s">
-        <v>238</v>
-      </c>
-      <c r="F36" s="6" t="s">
-        <v>239</v>
-      </c>
-      <c r="G36" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="H36" s="6" t="s">
-        <v>169</v>
-      </c>
-      <c r="I36" s="6" t="s">
-        <v>240</v>
-      </c>
-      <c r="J36" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="K36" s="6" t="s">
-        <v>246</v>
-      </c>
-      <c r="L36" s="6" t="s">
-        <v>242</v>
-      </c>
-      <c r="M36" s="6" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="37" spans="1:13" ht="29" x14ac:dyDescent="0.35">
-      <c r="A37" s="6" t="s">
-        <v>193</v>
-      </c>
-      <c r="B37" s="6" t="s">
-        <v>235</v>
-      </c>
-      <c r="C37" s="6" t="s">
-        <v>247</v>
-      </c>
-      <c r="D37" s="6" t="s">
-        <v>248</v>
-      </c>
-      <c r="E37" s="6" t="s">
-        <v>238</v>
-      </c>
-      <c r="F37" s="6" t="s">
-        <v>239</v>
-      </c>
-      <c r="G37" s="6" t="s">
-        <v>227</v>
-      </c>
-      <c r="H37" s="6" t="s">
-        <v>249</v>
-      </c>
-      <c r="I37" s="6" t="s">
-        <v>250</v>
-      </c>
-      <c r="J37" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="K37" s="6" t="s">
-        <v>251</v>
-      </c>
-      <c r="L37" s="6" t="s">
-        <v>242</v>
-      </c>
-      <c r="M37" s="6" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="38" spans="1:13" ht="29" x14ac:dyDescent="0.35">
-      <c r="A38" s="8" t="s">
-        <v>252</v>
-      </c>
-      <c r="B38" s="8" t="s">
-        <v>253</v>
-      </c>
-      <c r="C38" s="8" t="s">
-        <v>253</v>
-      </c>
-      <c r="D38" s="8" t="s">
-        <v>254</v>
-      </c>
-      <c r="E38" s="8" t="s">
-        <v>255</v>
-      </c>
-      <c r="F38" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="G38" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="H38" s="8" t="s">
-        <v>256</v>
-      </c>
-      <c r="I38" s="8" t="s">
-        <v>148</v>
-      </c>
-      <c r="J38" s="8" t="s">
-        <v>257</v>
-      </c>
-      <c r="K38" s="8" t="s">
-        <v>258</v>
-      </c>
-      <c r="L38" s="8" t="s">
+      <c r="K42" s="7" t="s">
+        <v>275</v>
+      </c>
+      <c r="L42" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="M38" s="8" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A39" s="8" t="s">
-        <v>252</v>
-      </c>
-      <c r="B39" s="8" t="s">
-        <v>260</v>
-      </c>
-      <c r="C39" s="8" t="s">
-        <v>261</v>
-      </c>
-      <c r="D39" s="8" t="s">
-        <v>262</v>
-      </c>
-      <c r="E39" s="8" t="s">
-        <v>103</v>
-      </c>
-      <c r="F39" s="8" t="s">
-        <v>122</v>
-      </c>
-      <c r="G39" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="H39" s="8" t="s">
-        <v>263</v>
-      </c>
-      <c r="I39" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="J39" s="8" t="s">
-        <v>257</v>
-      </c>
-      <c r="K39" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="L39" s="8" t="s">
-        <v>124</v>
-      </c>
-      <c r="M39" s="8" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="40" spans="1:13" ht="29" x14ac:dyDescent="0.35">
-      <c r="A40" s="8" t="s">
-        <v>252</v>
-      </c>
-      <c r="B40" s="8" t="s">
-        <v>264</v>
-      </c>
-      <c r="C40" s="8" t="s">
-        <v>265</v>
-      </c>
-      <c r="D40" s="8" t="s">
-        <v>266</v>
-      </c>
-      <c r="E40" s="8" t="s">
-        <v>267</v>
-      </c>
-      <c r="F40" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="G40" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="H40" s="8" t="s">
-        <v>268</v>
-      </c>
-      <c r="I40" s="8" t="s">
-        <v>148</v>
-      </c>
-      <c r="J40" s="8" t="s">
-        <v>257</v>
-      </c>
-      <c r="K40" s="8" t="s">
-        <v>269</v>
-      </c>
-      <c r="L40" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="M40" s="8" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="41" spans="1:13" ht="29" x14ac:dyDescent="0.35">
-      <c r="A41" s="8" t="s">
-        <v>252</v>
-      </c>
-      <c r="B41" s="8" t="s">
-        <v>271</v>
-      </c>
-      <c r="C41" s="8" t="s">
-        <v>271</v>
-      </c>
-      <c r="D41" s="8" t="s">
-        <v>272</v>
-      </c>
-      <c r="E41" s="8" t="s">
-        <v>255</v>
-      </c>
-      <c r="F41" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="G41" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="H41" s="8" t="s">
-        <v>273</v>
-      </c>
-      <c r="I41" s="8" t="s">
-        <v>274</v>
-      </c>
-      <c r="J41" s="8" t="s">
-        <v>257</v>
-      </c>
-      <c r="K41" s="8" t="s">
-        <v>258</v>
-      </c>
-      <c r="L41" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="M41" s="8" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="42" spans="1:13" ht="29" x14ac:dyDescent="0.35">
-      <c r="A42" s="8" t="s">
-        <v>252</v>
-      </c>
-      <c r="B42" s="8" t="s">
-        <v>275</v>
-      </c>
-      <c r="C42" s="8" t="s">
-        <v>275</v>
-      </c>
-      <c r="D42" s="8" t="s">
+      <c r="M42" s="7" t="s">
         <v>276</v>
       </c>
-      <c r="E42" s="8" t="s">
-        <v>255</v>
-      </c>
-      <c r="F42" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="G42" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="H42" s="8" t="s">
-        <v>277</v>
-      </c>
-      <c r="I42" s="8" t="s">
-        <v>274</v>
-      </c>
-      <c r="J42" s="8" t="s">
-        <v>257</v>
-      </c>
-      <c r="K42" s="8" t="s">
-        <v>258</v>
-      </c>
-      <c r="L42" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="M42" s="8" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="43" spans="1:13" ht="29" x14ac:dyDescent="0.35">
-      <c r="A43" s="8" t="s">
-        <v>252</v>
-      </c>
-      <c r="B43" s="8" t="s">
-        <v>278</v>
-      </c>
-      <c r="C43" s="8" t="s">
-        <v>278</v>
-      </c>
-      <c r="D43" s="8" t="s">
-        <v>279</v>
-      </c>
-      <c r="E43" s="8" t="s">
-        <v>255</v>
-      </c>
-      <c r="F43" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="G43" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="H43" s="8" t="s">
-        <v>280</v>
-      </c>
-      <c r="I43" s="8" t="s">
-        <v>281</v>
-      </c>
-      <c r="J43" s="8" t="s">
-        <v>257</v>
-      </c>
-      <c r="K43" s="8" t="s">
-        <v>258</v>
-      </c>
-      <c r="L43" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="M43" s="8" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="44" spans="1:13" ht="29" x14ac:dyDescent="0.35">
-      <c r="A44" s="8" t="s">
-        <v>252</v>
-      </c>
-      <c r="B44" s="8" t="s">
-        <v>282</v>
-      </c>
-      <c r="C44" s="8" t="s">
-        <v>282</v>
-      </c>
-      <c r="D44" s="8" t="s">
-        <v>283</v>
-      </c>
-      <c r="E44" s="8" t="s">
-        <v>255</v>
-      </c>
-      <c r="F44" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="G44" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="H44" s="8" t="s">
-        <v>284</v>
-      </c>
-      <c r="I44" s="8" t="s">
-        <v>285</v>
-      </c>
-      <c r="J44" s="8" t="s">
-        <v>257</v>
-      </c>
-      <c r="K44" s="8" t="s">
-        <v>258</v>
-      </c>
-      <c r="L44" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="M44" s="8" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="45" spans="1:13" ht="29" x14ac:dyDescent="0.35">
-      <c r="A45" s="8" t="s">
-        <v>252</v>
-      </c>
-      <c r="B45" s="8" t="s">
-        <v>287</v>
-      </c>
-      <c r="C45" s="8" t="s">
-        <v>287</v>
-      </c>
-      <c r="D45" s="8" t="s">
-        <v>288</v>
-      </c>
-      <c r="E45" s="8" t="s">
-        <v>255</v>
-      </c>
-      <c r="F45" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="G45" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="H45" s="8" t="s">
-        <v>289</v>
-      </c>
-      <c r="I45" s="8" t="s">
-        <v>285</v>
-      </c>
-      <c r="J45" s="8" t="s">
-        <v>257</v>
-      </c>
-      <c r="K45" s="8" t="s">
-        <v>258</v>
-      </c>
-      <c r="L45" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="M45" s="8" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A46" s="8" t="s">
-        <v>252</v>
-      </c>
-      <c r="B46" s="8" t="s">
-        <v>290</v>
-      </c>
-      <c r="C46" s="8" t="s">
-        <v>290</v>
-      </c>
-      <c r="D46" s="8" t="s">
-        <v>291</v>
-      </c>
-      <c r="E46" s="8" t="s">
-        <v>292</v>
-      </c>
-      <c r="F46" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="G46" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="H46" s="8" t="s">
-        <v>293</v>
-      </c>
-      <c r="I46" s="8" t="s">
-        <v>240</v>
-      </c>
-      <c r="J46" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="K46" s="8" t="s">
-        <v>294</v>
-      </c>
-      <c r="L46" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="M46" s="8" t="s">
-        <v>295</v>
-      </c>
-    </row>
-    <row r="47" spans="1:13" ht="29" x14ac:dyDescent="0.35">
-      <c r="A47" s="8" t="s">
-        <v>252</v>
-      </c>
-      <c r="B47" s="8" t="s">
-        <v>235</v>
-      </c>
-      <c r="C47" s="8" t="s">
-        <v>296</v>
-      </c>
-      <c r="D47" s="8" t="s">
-        <v>297</v>
-      </c>
-      <c r="E47" s="8" t="s">
-        <v>238</v>
-      </c>
-      <c r="F47" s="8" t="s">
-        <v>239</v>
-      </c>
-      <c r="G47" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="H47" s="8" t="s">
-        <v>298</v>
-      </c>
-      <c r="I47" s="8" t="s">
-        <v>299</v>
-      </c>
-      <c r="J47" s="8" t="s">
-        <v>257</v>
-      </c>
-      <c r="K47" s="8" t="s">
-        <v>300</v>
-      </c>
-      <c r="L47" s="8" t="s">
-        <v>242</v>
-      </c>
-      <c r="M47" s="8" t="s">
-        <v>301</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M47" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:M42"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="16.7265625" customWidth="1"/>
-    <col min="2" max="2" width="72.7265625" customWidth="1"/>
+    <col min="1" max="1" width="16.7109375" customWidth="1"/>
+    <col min="2" max="2" width="72.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>302</v>
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>303</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
       <c r="A2" s="2" t="s">
         <v>13</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>304</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
       <c r="A3" s="3" t="s">
         <v>49</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>305</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
       <c r="A4" s="5" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>306</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
       <c r="A5" s="6" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A6" s="8" t="s">
-        <v>252</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A7" s="7" t="s">
-        <v>309</v>
-      </c>
-      <c r="B7" s="7" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A8" s="4" t="s">
-        <v>311</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>312</v>
+        <v>281</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" s="7" t="s">
+        <v>237</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>284</v>
       </c>
     </row>
   </sheetData>

</xml_diff>